<commit_message>
work types (admin-managed, isPlanning) replace invoice kind enum; project types: Fiberization, خدمة شاملة, FTTS, إتاحة, Closed Compound; template 02 gains work types sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/02_المشروعات.xlsx
+++ b/apps/web/public/templates/02_المشروعات.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أنواع المشروعات" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المشروعات" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="أنواع الأعمال" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المشروعات" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تعليمات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="5" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -555,24 +556,24 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>FTTH</t>
+          <t>FIBERIZATION</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>FTTH — ألياف للمنازل</t>
+          <t>Fiberization</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>MSAN</t>
+          <t>ACCESS</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>إحلال كابينات MSAN</t>
+          <t>إتاحة</t>
         </is>
       </c>
     </row>
@@ -582,6 +583,81 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>كود نوع الأعمال *</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>نوع الأعمال *</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>مستخلص تخطيط؟</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>is_planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CIVIL_MAINT</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>صيانة مدني</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>لا</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C3:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="اختار من القائمة" type="list">
+      <formula1>"نعم,لا"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -675,7 +751,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>FTTH</t>
+          <t>FIBERIZATION</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1584,13 +1660,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1606,7 +1682,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>الغرض: تعريف أنواع المشروعات والمشروعات وربط كل مشروع بالسنترال.</t>
+          <t>الغرض: تعريف أنواع المشروعات وأنواع الأعمال والمشروعات وربط كل مشروع بالسنترال.</t>
         </is>
       </c>
     </row>
@@ -1642,54 +1718,78 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr"/>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>• شيت أنواع الأعمال اختياري — الأنواع الأساسية متسجلة في المنظومة، وتقدر تضيف غيرها هنا أو من شاشة الهيكل.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>قواعد عامة لكل القوالب</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>• ما تغيّرش أسماء الشيتات ولا ترتيب الأعمدة ولا الصف التاني (اسم العمود التقني).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>• العمود اللي عليه * إلزامي. الأعمدة اللي فيها قائمة لازم تختار منها.</t>
+          <t>• ما تغيّرش أسماء الشيتات ولا ترتيب الأعمدة ولا الصف التاني (اسم العمود التقني).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>• الصفوف الرمادي أمثلة — امسحها قبل الرفع.</t>
+          <t>• العمود اللي عليه * إلزامي. الأعمدة اللي فيها قائمة لازم تختار منها.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>• الأرقام من غير فواصل أو عملة. التواريخ يوم/شهر/سنة.</t>
+          <t>• الصفوف الرمادي أمثلة — امسحها قبل الرفع.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
+          <t>• الأرقام من غير فواصل أو عملة. التواريخ يوم/شهر/سنة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
           <t>• عند الرفع السيستم بيعرض معاينة بكل صف وأخطاؤه قبل الحفظ — مفيش حاجة بتتحفظ قبل ما توافق.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>• نسخة القالب: 1.0 — لو القالب قديم السيستم هيطلب تنزيل النسخة الجديدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>شرح الأعمدة</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>• [أنواع الأعمال] مستخلص تخطيط؟: نعم = بيتصرف 100% بعد الانتهاء من غير محجوز As-Built ولا تسليم</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1739,7 +1839,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"أنواع المشروعات": [["FTTH", "FTTH — ألياف للمنازل"], ["MSAN", "إحلال كابينات MSAN"]], "المشروعات": [["PJ-RABAA", "حى الحدق — سنترال رابعة", "FTTH", "C-RABAA", "", ""]]}</t>
+          <t>{"أنواع المشروعات": [["FIBERIZATION", "Fiberization"], ["ACCESS", "إتاحة"]], "أنواع الأعمال": [["CIVIL_MAINT", "صيانة مدني", "لا"]], "المشروعات": [["PJ-RABAA", "حى الحدق — سنترال رابعة", "FIBERIZATION", "C-RABAA", "", ""]]}</t>
         </is>
       </c>
     </row>

</xml_diff>